<commit_message>
Update arm parameters workbook and add phase 1B reducer and output encoder bench documentation
</commit_message>
<xml_diff>
--- a/docs/arm-parameters.xlsx
+++ b/docs/arm-parameters.xlsx
@@ -543,7 +543,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Change confirmed design values in the generator and regenerate. Add raw observations and measured outputs directly to Test Log; regeneration preserves its existing rows.</t>
+          <t>Change confirmed design values in the generator and regenerate. Add raw observations and measured outputs directly to Test Log; regeneration preserves all existing rows.</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1410,7 +1410,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Phase 1B Reducer Bill of Materials</t>
+          <t>Phase 1 Reducer and Control Electronics BOM</t>
         </is>
       </c>
     </row>
@@ -1454,167 +1454,177 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Output</t>
+          <t>Control</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Main bearing</t>
+          <t>Microcontroller</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>6705-2RS</t>
+          <t>Arduino Uno</t>
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Selected</t>
+          <t>On hand</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Supports output flanges</t>
+          <t>Phase 1 step generation and I2C control</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Flange land 25 mm; axial lip</t>
+          <t>Elegoo starter kit</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Cycloidal</t>
+          <t>Motor control</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Disc-center bearing</t>
+          <t>Stepper driver</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>MR148ZZ</t>
+          <t>TMC2209 StepStick module</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Selected</t>
+          <t>On hand</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Supports cycloidal disc center bore</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
+          <t>NEMA 17 step/dir drive</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Heatsink fitted; Vref/current to verify</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Sensing</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Crankshaft bearing</t>
+          <t>Absolute encoder</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>687ZZ</t>
+          <t>AS5600 magnetic encoder breakout</t>
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Selected</t>
+          <t>On hand</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Supports PETG crankshaft in output flanges</t>
+          <t>Output-side joint angle</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Light press</t>
+          <t>First test wires directly to Uno I2C</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Cycloidal</t>
+          <t>Sensing</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Cycloidal discs</t>
+          <t>I2C mux</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>PETG, 15 lobes, 4 mm</t>
+          <t>TCA9548A breakout, address 0x70</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>On hand</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>15:1 stage; 180 deg indexed</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
+          <t>Separates multiple AS5600 encoders with shared address 0x36</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Not needed for one direct-wired encoder; required from joint 2</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Cycloidal</t>
+          <t>Power</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Integral ring pins</t>
+          <t>DC-DC converter</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>PETG, 3.5 mm diameter</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>16</v>
+          <t>5 V buck converter</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>On hand</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Fixed ring; side-embedded in housing</t>
+          <t>Regulated logic/encoder supply when required</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>CAD root geometry pending</t>
+          <t>Record selected module, input, and output voltage before use</t>
         </is>
       </c>
     </row>
@@ -1626,60 +1636,60 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Output shafts</t>
+          <t>Main bearing</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>M3 shoulder bolt, 4 mm shoulder</t>
+          <t>6705-2RS</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Procure</t>
+          <t>Selected</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Transfers disc motion; retains core</t>
+          <t>Supports output flanges</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>23 mm diameter circle</t>
+          <t>Flange land 25 mm; axial lip</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Output</t>
+          <t>Cycloidal</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>PTFE spacer</t>
+          <t>Disc-center bearing</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>0.8 mm</t>
+          <t>MR148ZZ</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Procure</t>
+          <t>Selected</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Disc-to-flange separation</t>
+          <t>Supports cycloidal disc center bore</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr"/>
@@ -1687,93 +1697,87 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Interface</t>
+          <t>Input</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Link inserts</t>
+          <t>Crankshaft bearing</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>M3 heat-set insert</t>
+          <t>687ZZ</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Procure</t>
+          <t>Selected</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Linkage connection</t>
+          <t>Supports PETG crankshaft in output flanges</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>16 mm diameter circle</t>
+          <t>Light press</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Fasteners</t>
+          <t>Cycloidal</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Internal fasteners</t>
+          <t>Cycloidal discs</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
+          <t>PETG, 15 lobes, 4 mm</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Procure</t>
+          <t>Print</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Reducer assembly</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Lengths pending flange design</t>
-        </is>
-      </c>
+          <t>15:1 stage; 180 deg indexed</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Input</t>
+          <t>Cycloidal</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Crankshaft</t>
+          <t>Integral ring pins</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>PETG, NEMA 17 shaft-flat drive</t>
+          <t>PETG, 3.5 mm diameter</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -1782,76 +1786,249 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Eccentric input</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr"/>
+          <t>Fixed ring; side-embedded in housing</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>CAD root geometry pending</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Encoder</t>
+          <t>Output</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Encoder</t>
+          <t>Output shafts</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>AS5600 absolute magnetic</t>
+          <t>M3 shoulder bolt, 4 mm shoulder</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>On hand</t>
+          <t>Procure</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Output-side joint angle</t>
+          <t>Transfers disc motion; retains core</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Magnet and gap pending</t>
+          <t>23 mm diameter circle</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>Output</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>PTFE spacer</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>0.8 mm</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Procure</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Disc-to-flange separation</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Interface</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Link inserts</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>M3 heat-set insert</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Procure</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Linkage connection</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>16 mm diameter circle</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Fasteners</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Internal fasteners</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Procure</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Reducer assembly</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Lengths pending flange design</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Crankshaft</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>PETG, NEMA 17 shaft-flat drive</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Print</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Eccentric input</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Encoder</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Encoder</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>AS5600 absolute magnetic</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>On hand</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Output-side joint angle</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Magnet and gap pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>Lubrication</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Grease</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Super Lube Multi-Purpose Synthetic</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D20" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>On hand</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>Run-in and friction reduction</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Coupon compatibility test pending</t>
         </is>
@@ -11891,7 +12068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11960,7 +12137,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Unpowered, ungreased then lightly greased</t>
+          <t>Unpowered, before then after light grease</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -11980,7 +12157,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Never power a binding reducer</t>
+          <t>Repeat whenever assembly changes</t>
         </is>
       </c>
     </row>
@@ -11992,32 +12169,32 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Unloaded run-in</t>
+          <t>Output encoder by hand</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Driver current/Vref, input RPM, duration, direction</t>
+          <t>Magnet gap and output rotation</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Temperature, current, noise, resistance before/after</t>
+          <t>AGC, magnet state, 360 deg continuity</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>10-15 min each direction; stop on binding or rapid heat</t>
+          <t>No status loss or angle jumps</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Wipe plastic debris before final grease</t>
+          <t>Run app_01_encoder_test before motor power</t>
         </is>
       </c>
     </row>
@@ -12029,22 +12206,22 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Actual ratio</t>
+          <t>Direct-step reducer inspection</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Mark input/output; count input turns</t>
+          <t>app_10_reducer_bench; 160 then 1600 motor-step jogs</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Input turns per output turn</t>
+          <t>Output direction, AS5600 motion, noise, I2C errors</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Measured value becomes firmware GEAR_RATIO</t>
+          <t>No binding, heat, or encoder fault</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -12054,7 +12231,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Do not use nominal 15:1 without this</t>
+          <t>GEAR_RATIO intentionally unused</t>
         </is>
       </c>
     </row>
@@ -12066,22 +12243,22 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Backlash</t>
+          <t>Unloaded run-in</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Output vertical or counterbalanced; 100 mm lever</t>
+          <t>Verified driver current, input RPM, duration, direction</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Dial displacement and AS5600 angle, both directions</t>
+          <t>Temperature, current, noise, resistance before/after</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Report degrees and repeatability</t>
+          <t>10-15 min each direction; stop on binding or rapid heat</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -12091,7 +12268,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Avoid gravity preload masking backlash</t>
+          <t>Wipe plastic debris before final grease</t>
         </is>
       </c>
     </row>
@@ -12103,22 +12280,22 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Static stiffness</t>
+          <t>Actual ratio</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Known mass, lever radius, direction</t>
+          <t>Mark input/output; count input turns</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Torque, AS5600 deflection, residual after unload</t>
+          <t>Input turns per output turn</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Calculate k = torque / deflection</t>
+          <t>Measured value becomes firmware GEAR_RATIO</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -12128,7 +12305,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Inspect integrated pin-wall opening</t>
+          <t>Do not use nominal 15:1 without this</t>
         </is>
       </c>
     </row>
@@ -12140,22 +12317,22 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Efficiency / pullout</t>
+          <t>Backlash</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Current, motor speed, lever radius, fish-scale force</t>
+          <t>Output vertical or counterbalanced; 100 mm lever</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Output torque at stall, motor temperature</t>
+          <t>Dial displacement and AS5600 angle, both directions</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Compare to motor torque x ratio</t>
+          <t>Report degrees and repeatability</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -12165,7 +12342,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Start unloaded; test at conservative current</t>
+          <t>Avoid gravity preload masking backlash</t>
         </is>
       </c>
     </row>
@@ -12177,22 +12354,22 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>PETG grease coupon</t>
+          <t>Static stiffness</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Bent PETG coupon, Super Lube exposure</t>
+          <t>Known mass, lever radius, direction</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Crazing, crack, stiffness change after 12 h</t>
+          <t>Torque, AS5600 deflection, residual after unload</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>No visible craze or embrittlement</t>
+          <t>Calculate k = torque / deflection</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -12202,7 +12379,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Test at disc print settings</t>
+          <t>Inspect integrated pin-wall opening</t>
         </is>
       </c>
     </row>
@@ -12214,32 +12391,69 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Encoder under motion</t>
+          <t>Efficiency / pullout</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Magnet gap, speed, driver current</t>
+          <t>Current, motor speed, lever radius, fish-scale force</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>AS5600 status, I2C errors, encoder noise</t>
+          <t>Output torque at stall, motor temperature</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>No encoder loss during stepped motion</t>
+          <t>Compare to motor torque x ratio</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Mechanical encoder details pending</t>
+          <t>Start unloaded; test at conservative current</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>P1B-09</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>PETG grease coupon</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Bent PETG coupon, Super Lube exposure</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Crazing, crack, stiffness change after 12 h</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>No visible craze or embrittlement</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Test at disc print settings</t>
         </is>
       </c>
     </row>
@@ -12248,7 +12462,7 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="F4:F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F4:F12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Planned,Running,Pass,Fail,Blocked,Pending"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12262,7 +12476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12322,6 +12536,43 @@
       <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Enter a new row for each run; keep serial CSV files in docs/test-results/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>P1A-01</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Uno + TMC2209 + NEMA 17; 8x microstep; no encoder or reducer</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>12 V PSU, about 1 A limit; 900 / 1066 / 1600 steps/s</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Smooth at all tested rates after current adjustment; motor and driver cold</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>docs/test-results/2026-08-31-open-loop-motor-bench.txt</t>
         </is>
       </c>
     </row>

</xml_diff>